<commit_message>
Add Approval Matrix flow diagram banner; switch font to TH Sarabun New
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MFZG9sH6okPTrq3ntpn1iY
</commit_message>
<xml_diff>
--- a/Approval_Matrix_Survey.xlsx
+++ b/Approval_Matrix_Survey.xlsx
@@ -39,166 +39,166 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <i val="1"/>
       <color rgb="001F3864"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00595959"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00595959"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00548235"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00548235"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="007030A0"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="007030A0"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="007F6000"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <b val="1"/>
       <color rgb="007F6000"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Tahoma"/>
+      <name val="TH Sarabun New"/>
       <color rgb="00595959"/>
       <sz val="9"/>
     </font>
@@ -560,7 +560,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
       </font>
       <fill>
@@ -572,7 +572,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
       </font>
       <fill>
@@ -584,7 +584,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
         <color rgb="009C0006"/>
       </font>
@@ -597,7 +597,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
         <color rgb="007F6000"/>
       </font>
@@ -610,7 +610,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
         <color rgb="00375623"/>
       </font>
@@ -623,14 +623,14 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
         <color rgb="00C00000"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
         <color rgb="007F6000"/>
       </font>
@@ -653,7 +653,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
       </font>
       <fill>
@@ -665,21 +665,21 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
         <color rgb="00375623"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <b val="1"/>
         <color rgb="00C55A11"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="TH Sarabun New"/>
         <strike val="1"/>
         <color rgb="00A6A6A6"/>
       </font>

</xml_diff>

<commit_message>
Move flow diagram from unit sheets to the guide page only
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MFZG9sH6okPTrq3ntpn1iY
</commit_message>
<xml_diff>
--- a/Approval_Matrix_Survey.xlsx
+++ b/Approval_Matrix_Survey.xlsx
@@ -16,10 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'1_บริหารทั่วไป'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'2_ยุทธศาสตร์และแผน'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'3_วิจัยและบริการวิชาการ'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'4_การศึกษาและนักศึกษา'!$4:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'1_บริหารทั่วไป'!$4:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'2_ยุทธศาสตร์และแผน'!$4:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'3_วิจัยและบริการวิชาการ'!$4:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'4_การศึกษาและนักศึกษา'!$4:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -790,7 +790,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!D12</f>
+              <f>'Dashboard'!D20</f>
             </strRef>
           </tx>
           <spPr>
@@ -803,12 +803,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$13:$A$16</f>
+              <f>'Dashboard'!$A$21:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$D$13:$D$16</f>
+              <f>'Dashboard'!$D$21:$D$24</f>
             </numRef>
           </val>
         </ser>
@@ -817,7 +817,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!E12</f>
+              <f>'Dashboard'!E20</f>
             </strRef>
           </tx>
           <spPr>
@@ -830,12 +830,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$13:$A$16</f>
+              <f>'Dashboard'!$A$21:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$E$13:$E$16</f>
+              <f>'Dashboard'!$E$21:$E$24</f>
             </numRef>
           </val>
         </ser>
@@ -844,7 +844,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!F12</f>
+              <f>'Dashboard'!F20</f>
             </strRef>
           </tx>
           <spPr>
@@ -857,12 +857,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$13:$A$16</f>
+              <f>'Dashboard'!$A$21:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$F$13:$F$16</f>
+              <f>'Dashboard'!$F$21:$F$24</f>
             </numRef>
           </val>
         </ser>
@@ -871,7 +871,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!G12</f>
+              <f>'Dashboard'!G20</f>
             </strRef>
           </tx>
           <spPr>
@@ -884,12 +884,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$13:$A$16</f>
+              <f>'Dashboard'!$A$21:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$G$13:$G$16</f>
+              <f>'Dashboard'!$G$21:$G$24</f>
             </numRef>
           </val>
         </ser>
@@ -1005,12 +1005,12 @@
           </dPt>
           <cat>
             <numRef>
-              <f>'Dashboard'!$D$12:$G$12</f>
+              <f>'Dashboard'!$D$20:$G$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$D$17:$G$17</f>
+              <f>'Dashboard'!$D$25:$G$25</f>
             </numRef>
           </val>
         </ser>
@@ -1060,7 +1060,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!L12</f>
+              <f>'Dashboard'!L20</f>
             </strRef>
           </tx>
           <spPr>
@@ -1073,12 +1073,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$13:$A$16</f>
+              <f>'Dashboard'!$A$21:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$L$13:$L$16</f>
+              <f>'Dashboard'!$L$21:$L$24</f>
             </numRef>
           </val>
         </ser>
@@ -1087,7 +1087,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!M12</f>
+              <f>'Dashboard'!M20</f>
             </strRef>
           </tx>
           <spPr>
@@ -1100,12 +1100,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$13:$A$16</f>
+              <f>'Dashboard'!$A$21:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$M$13:$M$16</f>
+              <f>'Dashboard'!$M$21:$M$24</f>
             </numRef>
           </val>
         </ser>
@@ -1114,7 +1114,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!N12</f>
+              <f>'Dashboard'!N20</f>
             </strRef>
           </tx>
           <spPr>
@@ -1127,12 +1127,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$13:$A$16</f>
+              <f>'Dashboard'!$A$21:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$N$13:$N$16</f>
+              <f>'Dashboard'!$N$21:$N$24</f>
             </numRef>
           </val>
         </ser>
@@ -1179,7 +1179,37 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15240000" cy="2667000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6120000" cy="3060000"/>
@@ -1201,7 +1231,7 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3960000" cy="3060000"/>
@@ -1223,7 +1253,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>45</row>
+      <row>53</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6120000" cy="3060000"/>
@@ -1239,6 +1269,31 @@
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15240000" cy="2667000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -1534,7 +1589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1549,272 +1604,281 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="2" ht="27" customHeight="1"/>
+    <row r="3" ht="27" customHeight="1"/>
+    <row r="4" ht="27" customHeight="1"/>
+    <row r="5" ht="27" customHeight="1"/>
+    <row r="6" ht="27" customHeight="1"/>
+    <row r="7" ht="27" customHeight="1"/>
+    <row r="8" ht="27" customHeight="1"/>
+    <row r="9" ht="27" customHeight="1"/>
+    <row r="10" ht="27" customHeight="1"/>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>วัตถุประสงค์</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>ทบทวนว่ากระบวนการใดควร คง / ตัด การกลั่นกรองผ่านเลขานุการคณะ (D2) หรือเปลี่ยนให้หน่วยงานผู้เชี่ยวชาญตรวจแทน โดยใช้ข้อมูลจริงจากหัวหน้างาน เพื่อลดขั้นตอนและ Lead Time โดยยังคงการควบคุมภายในให้สอดคล้องกับระดับความเสี่ยง</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>ระดับในสาย Approval</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ระดับ</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>ตำแหน่ง</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>บทบาทหลัก</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>ผู้ปฏิบัติ</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>เจ้าของเรื่อง จัดทำข้อมูล เอกสาร และรายละเอียดเพื่อเสนอขออนุมัติ</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>หัวหน้างาน</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>ควบคุมงานประจำ รับรองความถูกต้องและความจำเป็นของงาน</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>เลขานุการคณะ</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>กำกับดูแลภาพรวมสำนักงาน กลั่นกรองเรื่องที่มีความเสี่ยงหรือกระทบหลายหน่วยงาน  ◀ จุดที่สำรวจ</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>หน่วยงานเฉพาะทาง</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>กำกับดูแลระเบียบ ข้อบังคับ มาตรฐาน หรือความถูกต้องทางวิชาชีพในเรื่องนั้นโดยเฉพาะ</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>รองคณบดี</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>พิจารณาอนุมัติในสายงานที่กำกับดูแล</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>คณบดี</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>อนุมัติเรื่องสำคัญของคณะ มีผลผูกพันด้านงบประมาณ นโยบาย หรือทรัพยากร</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>มหาวิทยาลัย/อธิการบดี/สภา</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>อนุมัติเรื่องที่เกินอำนาจคณะ หรือเป็นไปตามข้อบังคับมหาวิทยาลัย</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>วิธีกรอก (ใช้เวลาประมาณ 30–60 นาทีต่อหน่วยงาน)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>1. เปิดชีตของหน่วยงานตนเอง (ชื่อชีตขึ้นต้นด้วยเลข 1–4) — รายการกระบวนการตั้งต้น 42 รายการ ทุกงานต้องตอบครบทุกรายการ</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>2. กรอกช่องสีเหลืองอ่อนทีละแถว: จำนวนรายการต่อปี, ระยะเวลาเฉลี่ย (วัน), ระยะเวลาที่ D2 ใช้ (วัน)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>3. ประเมินผลกระทบ 6 ด้านด้วย Yes/No และประเมินการควบคุม (มีผู้เชี่ยวชาญตรวจอยู่แล้วหรือไม่ / D2 เพิ่มคุณค่า / D2 เคยตีกลับ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>4. เลือก 'ข้อเสนอของหัวหน้างาน' — ถ้าเลือก 'เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ' ต้องเลือกหน่วยงานในช่องถัดไปด้วย</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>5. ถ้ากระบวนการใดไม่เคยเกิดขึ้นในงานของท่าน ให้ใส่จำนวนรายการต่อปีเป็น 0 (แถวจะเป็นสีเทาขีดฆ่า และไม่ถูกนับใน Dashboard) ไม่ต้องกรอกช่องอื่น</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>6. มีกระบวนการเพิ่มเติม: เพิ่มชื่อในแถวว่างด้านล่างของตาราง (สูตรและ Dropdown เตรียมไว้แล้ว)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>7. ดูช่อง 'ธงเตือน' — ถ้ามีข้อความ แสดงว่าข้อเสนอขัดกับระดับความเสี่ยง ควรทบทวนหรือใส่เหตุผลในช่องข้อเสนอแนะ</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>วิธีคำนวณคะแนนความเสี่ยง (ค่าตั้งต้น ปรับได้ที่ชีต Settings)</t>
+          <t>วิธีกรอก (ใช้เวลาประมาณ 30–60 นาทีต่อหน่วยงาน)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>คะแนน = 25 × [งบประมาณ=Yes] + 25 × [อัตรากำลัง=Yes] + 25 × [กฎหมาย/ระเบียบ=Yes] + 25 × [ยังไม่มีผู้เชี่ยวชาญตรวจ (=No)]</t>
+          <t>1. เปิดชีตของหน่วยงานตนเอง (ชื่อชีตขึ้นต้นด้วยเลข 1–4) — รายการกระบวนการตั้งต้น 42 รายการ ทุกงานต้องตอบครบทุกรายการ</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>ระดับ: ต่ำ = คะแนนน้อยกว่า 50   |   ปานกลาง = 50 ถึงน้อยกว่า 75   |   สูง = ตั้งแต่ 75</t>
+          <t>2. กรอกช่องสีเหลืองอ่อนทีละแถว: จำนวนรายการต่อปี, ระยะเวลาเฉลี่ย (วัน), ระยะเวลาที่ D2 ใช้ (วัน)</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>ผลกระทบด้านทรัพย์สิน/พัสดุ ชื่อเสียงองค์กร และนโยบาย เก็บเป็นข้อมูลประกอบ ไม่นำมาคิดคะแนนตามที่ Template กำหนด</t>
+          <t>3. ประเมินผลกระทบ 6 ด้านด้วย Yes/No และประเมินการควบคุม (มีผู้เชี่ยวชาญตรวจอยู่แล้วหรือไม่ / D2 เพิ่มคุณค่า / D2 เคยตีกลับ)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>4. เลือก 'ข้อเสนอของหัวหน้างาน' — ถ้าเลือก 'เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ' ต้องเลือกหน่วยงานในช่องถัดไปด้วย</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>5. ถ้ากระบวนการใดไม่เคยเกิดขึ้นในงานของท่าน ให้ใส่จำนวนรายการต่อปีเป็น 0 (แถวจะเป็นสีเทาขีดฆ่า และไม่ถูกนับใน Dashboard) ไม่ต้องกรอกช่องอื่น</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>6. มีกระบวนการเพิ่มเติม: เพิ่มชื่อในแถวว่างด้านล่างของตาราง (สูตรและ Dropdown เตรียมไว้แล้ว)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>7. ดูช่อง 'ธงเตือน' — ถ้ามีข้อความ แสดงว่าข้อเสนอขัดกับระดับความเสี่ยง ควรทบทวนหรือใส่เหตุผลในช่องข้อเสนอแนะ</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>วิธีคำนวณคะแนนความเสี่ยง (ค่าตั้งต้น ปรับได้ที่ชีต Settings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>คะแนน = 25 × [งบประมาณ=Yes] + 25 × [อัตรากำลัง=Yes] + 25 × [กฎหมาย/ระเบียบ=Yes] + 25 × [ยังไม่มีผู้เชี่ยวชาญตรวจ (=No)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>ระดับ: ต่ำ = คะแนนน้อยกว่า 50   |   ปานกลาง = 50 ถึงน้อยกว่า 75   |   สูง = ตั้งแต่ 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>ผลกระทบด้านทรัพย์สิน/พัสดุ ชื่อเสียงองค์กร และนโยบาย เก็บเป็นข้อมูลประกอบ ไม่นำมาคิดคะแนนตามที่ Template กำหนด</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t>Dashboard ไม่นับกระบวนการที่จำนวนรายการต่อปี = 0  |  ร้อยละคิดจากกระบวนการที่ตอบ 'ข้อเสนอของหัวหน้างาน' แล้ว  |  วันทำการที่ประหยัดได้ = จำนวนรายการต่อปี × ระยะเวลาที่ D2 ใช้ (เฉพาะแถวที่เสนอตัด D2)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>สีที่ใช้</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr"/>
-      <c r="B32" s="6" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr"/>
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>ช่องที่ต้องกรอก</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr"/>
-      <c r="B33" s="6" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr"/>
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>สูตรอัตโนมัติ / ข้อมูลตั้งต้น (ห้ามแก้)</t>
         </is>
@@ -1823,20 +1887,21 @@
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A38:C38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1847,7 +1912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A9:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1869,723 +1934,731 @@
     <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="27" customHeight="1"/>
+    <row r="2" ht="27" customHeight="1"/>
+    <row r="3" ht="27" customHeight="1"/>
+    <row r="4" ht="27" customHeight="1"/>
+    <row r="5" ht="27" customHeight="1"/>
+    <row r="6" ht="27" customHeight="1"/>
+    <row r="7" ht="27" customHeight="1"/>
+    <row r="8" ht="27" customHeight="1"/>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Dashboard สรุปผลสำรวจ Approval Matrix (Risk-Based Approval)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>สรุปอัตโนมัติจากชีตของหัวหน้างานทั้ง 4 งาน — ไม่นับกระบวนการที่ไม่เคยทำ (จำนวนรายการ = 0) และร้อยละคิดจากกระบวนการที่ตอบข้อเสนอแล้ว</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>⚠ หมายเหตุสำคัญ: ตัวเลข 'ระยะเวลาดำเนินการเฉลี่ย' / 'ระยะเวลาที่ D2 ใช้' และ 'วันทำการที่ประหยัดได้' เป็นค่าประมาณจากความทรงจำของหัวหน้างานแต่ละคน ไม่ใช่ข้อมูลที่ดึงจากระบบ eDoc จริง — ใช้ประกอบการพิจารณาทิศทาง (เช่น กระบวนการไหนน่าจะช้า) ไม่ควรใช้เป็นตัวเลขทางการที่แม่นยำ 100% ในการรายงานผู้บริหาร</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>เลือกหน่วยงานที่ต้องการดู ▶</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>ทั้งคณะ</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n"/>
-      <c r="D4" s="15" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>ภาพรวม</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="16" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>กระบวนการทั้งหมด</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>ตอบข้อเสนอแล้ว</t>
         </is>
       </c>
-      <c r="E7" s="19" t="n"/>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="20" t="inlineStr">
         <is>
           <t>เสนอให้ คง D2</t>
         </is>
       </c>
-      <c r="G7" s="21" t="n"/>
-      <c r="H7" s="22" t="inlineStr">
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>เสนอให้ ตัด D2</t>
         </is>
       </c>
-      <c r="I7" s="23" t="n"/>
-      <c r="J7" s="24" t="inlineStr">
+      <c r="I15" s="23" t="n"/>
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>เสนอให้เปลี่ยนเป็นผู้เชี่ยวชาญ</t>
         </is>
       </c>
-      <c r="K7" s="25" t="n"/>
-      <c r="L7" s="26" t="inlineStr">
+      <c r="K15" s="25" t="n"/>
+      <c r="L15" s="26" t="inlineStr">
         <is>
           <t>ขอหารือเพิ่มเติม</t>
         </is>
       </c>
-      <c r="M7" s="27" t="n"/>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="B8" s="28">
-        <f>INDEX($B$13:$B$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="D8" s="29">
-        <f>INDEX($C$13:$C$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="F8" s="30">
-        <f>INDEX($D$13:$D$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="H8" s="31">
-        <f>INDEX($E$13:$E$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="J8" s="32">
-        <f>INDEX($F$13:$F$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="L8" s="33">
-        <f>INDEX($G$13:$G$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="34">
-        <f>"หน่วยงาน: "&amp;$B$4</f>
-        <v/>
-      </c>
-      <c r="D9" s="35">
-        <f>IF(INDEX($B$13:$B$17,MATCH($B$4,$A$13:$A$17,0))=0,"",INDEX($C$13:$C$17,MATCH($B$4,$A$13:$A$17,0))/INDEX($B$13:$B$17,MATCH($B$4,$A$13:$A$17,0)))</f>
-        <v/>
-      </c>
-      <c r="F9" s="36">
-        <f>INDEX($H$13:$H$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="H9" s="37">
-        <f>INDEX($I$13:$I$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="J9" s="38">
-        <f>INDEX($J$13:$J$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-      <c r="L9" s="39">
-        <f>INDEX($K$13:$K$17,MATCH($B$4,$A$13:$A$17,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="40">
+      <c r="M15" s="27" t="n"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="B16" s="28">
+        <f>INDEX($B$21:$B$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="D16" s="29">
+        <f>INDEX($C$21:$C$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="F16" s="30">
+        <f>INDEX($D$21:$D$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="H16" s="31">
+        <f>INDEX($E$21:$E$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="J16" s="32">
+        <f>INDEX($F$21:$F$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="L16" s="33">
+        <f>INDEX($G$21:$G$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="34">
+        <f>"หน่วยงาน: "&amp;$B$12</f>
+        <v/>
+      </c>
+      <c r="D17" s="35">
+        <f>IF(INDEX($B$21:$B$25,MATCH($B$12,$A$21:$A$25,0))=0,"",INDEX($C$21:$C$25,MATCH($B$12,$A$21:$A$25,0))/INDEX($B$21:$B$25,MATCH($B$12,$A$21:$A$25,0)))</f>
+        <v/>
+      </c>
+      <c r="F17" s="36">
+        <f>INDEX($H$21:$H$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="H17" s="37">
+        <f>INDEX($I$21:$I$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="J17" s="38">
+        <f>INDEX($J$21:$J$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+      <c r="L17" s="39">
+        <f>INDEX($K$21:$K$25,MATCH($B$12,$A$21:$A$25,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="40">
         <f>"หมายเหตุ: ไม่นับกระบวนการที่ไม่เคยทำ (จำนวนรายการต่อปี = 0) รวม "&amp;(COUNTIFS('1_บริหารทั่วไป'!$C$7:$C$91,"?*",'1_บริหารทั่วไป'!$D$7:$D$91,0)+COUNTIFS('2_ยุทธศาสตร์และแผน'!$C$7:$C$91,"?*",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,0)+COUNTIFS('3_วิจัยและบริการวิชาการ'!$C$7:$C$91,"?*",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,0)+COUNTIFS('4_การศึกษาและนักศึกษา'!$C$7:$C$91,"?*",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,0))&amp;" รายการ"</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>ตารางสรุปแยกตามหน่วยงาน</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>หน่วยงาน</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>กระบวนการ
 ทั้งหมด</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>ตอบข้อเสนอ
 แล้ว</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>คง D2</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>ตัด D2</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>เปลี่ยนเป็น
 ผู้เชี่ยวชาญ</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>ขอหารือ
 เพิ่มเติม</t>
         </is>
       </c>
-      <c r="H12" s="16" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>% คง D2</t>
         </is>
       </c>
-      <c r="I12" s="16" t="inlineStr">
+      <c r="I20" s="16" t="inlineStr">
         <is>
           <t>% ตัด D2</t>
         </is>
       </c>
-      <c r="J12" s="16" t="inlineStr">
+      <c r="J20" s="16" t="inlineStr">
         <is>
           <t>% เปลี่ยน</t>
         </is>
       </c>
-      <c r="K12" s="16" t="inlineStr">
+      <c r="K20" s="16" t="inlineStr">
         <is>
           <t>% ขอหารือ</t>
         </is>
       </c>
-      <c r="L12" s="16" t="inlineStr">
+      <c r="L20" s="16" t="inlineStr">
         <is>
           <t>เสี่ยงสูง</t>
         </is>
       </c>
-      <c r="M12" s="16" t="inlineStr">
+      <c r="M20" s="16" t="inlineStr">
         <is>
           <t>เสี่ยงปานกลาง</t>
         </is>
       </c>
-      <c r="N12" s="16" t="inlineStr">
+      <c r="N20" s="16" t="inlineStr">
         <is>
           <t>เสี่ยงต่ำ</t>
         </is>
       </c>
-      <c r="O12" s="16" t="inlineStr">
+      <c r="O20" s="16" t="inlineStr">
         <is>
           <t>ธงเตือน</t>
         </is>
       </c>
-      <c r="P12" s="16" t="inlineStr">
+      <c r="P20" s="16" t="inlineStr">
         <is>
           <t>วันทำการที่
 ประหยัดได้/ปี</t>
         </is>
       </c>
-      <c r="Q12" s="16" t="inlineStr">
+      <c r="Q20" s="16" t="inlineStr">
         <is>
           <t>กรอกครบ
 (กระบวนการ)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="41" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>งานบริหารทั่วไป</t>
         </is>
       </c>
-      <c r="B13" s="42">
+      <c r="B21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$C$7:$C$91,"?*",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="C13" s="42">
+      <c r="C21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$C$7:$C$91,"?*",'1_บริหารทั่วไป'!$P$7:$P$91,"?*",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="D13" s="42">
+      <c r="D21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$P$7:$P$91,"คง D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="E13" s="42">
+      <c r="E21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$P$7:$P$91,"ตัด D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="F13" s="42">
+      <c r="F21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="G13" s="42">
+      <c r="G21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="H13" s="43">
-        <f>IF($C13=0,"",D13/$C13)</f>
-        <v/>
-      </c>
-      <c r="I13" s="43">
-        <f>IF($C13=0,"",E13/$C13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="43">
-        <f>IF($C13=0,"",F13/$C13)</f>
-        <v/>
-      </c>
-      <c r="K13" s="43">
-        <f>IF($C13=0,"",G13/$C13)</f>
-        <v/>
-      </c>
-      <c r="L13" s="42">
+      <c r="H21" s="43">
+        <f>IF($C21=0,"",D21/$C21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="43">
+        <f>IF($C21=0,"",E21/$C21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="43">
+        <f>IF($C21=0,"",F21/$C21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="43">
+        <f>IF($C21=0,"",G21/$C21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"สูง",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="M13" s="42">
+      <c r="M21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ปานกลาง",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="N13" s="42">
+      <c r="N21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ต่ำ",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="O13" s="42">
+      <c r="O21" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$T$7:$T$91,"?*",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="P13" s="44">
+      <c r="P21" s="44">
         <f>SUMIFS('1_บริหารทั่วไป'!$U$7:$U$91,'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="Q13" s="42">
+      <c r="Q21" s="42">
         <f>COUNTIF('1_บริหารทั่วไป'!$W$7:$W$91,"✔ ครบ")</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="41" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
         <is>
           <t>งานยุทธศาสตร์และแผน</t>
         </is>
       </c>
-      <c r="B14" s="42">
+      <c r="B22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$C$7:$C$91,"?*",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="C14" s="42">
+      <c r="C22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$C$7:$C$91,"?*",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"?*",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="D14" s="42">
+      <c r="D22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"คง D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="E14" s="42">
+      <c r="E22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ตัด D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="F14" s="42">
+      <c r="F22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="G14" s="42">
+      <c r="G22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="H14" s="43">
-        <f>IF($C14=0,"",D14/$C14)</f>
-        <v/>
-      </c>
-      <c r="I14" s="43">
-        <f>IF($C14=0,"",E14/$C14)</f>
-        <v/>
-      </c>
-      <c r="J14" s="43">
-        <f>IF($C14=0,"",F14/$C14)</f>
-        <v/>
-      </c>
-      <c r="K14" s="43">
-        <f>IF($C14=0,"",G14/$C14)</f>
-        <v/>
-      </c>
-      <c r="L14" s="42">
+      <c r="H22" s="43">
+        <f>IF($C22=0,"",D22/$C22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="43">
+        <f>IF($C22=0,"",E22/$C22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="43">
+        <f>IF($C22=0,"",F22/$C22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="43">
+        <f>IF($C22=0,"",G22/$C22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"สูง",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="M14" s="42">
+      <c r="M22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ปานกลาง",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="N14" s="42">
+      <c r="N22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ต่ำ",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="O14" s="42">
+      <c r="O22" s="42">
         <f>COUNTIFS('2_ยุทธศาสตร์และแผน'!$T$7:$T$91,"?*",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="P14" s="44">
+      <c r="P22" s="44">
         <f>SUMIFS('2_ยุทธศาสตร์และแผน'!$U$7:$U$91,'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="Q14" s="42">
+      <c r="Q22" s="42">
         <f>COUNTIF('2_ยุทธศาสตร์และแผน'!$W$7:$W$91,"✔ ครบ")</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="41" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="41" t="inlineStr">
         <is>
           <t>งานบริหารงานวิจัยและบริการวิชาการ</t>
         </is>
       </c>
-      <c r="B15" s="42">
+      <c r="B23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$C$7:$C$91,"?*",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="C15" s="42">
+      <c r="C23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$C$7:$C$91,"?*",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"?*",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="D15" s="42">
+      <c r="D23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"คง D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="E15" s="42">
+      <c r="E23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ตัด D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="F15" s="42">
+      <c r="F23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="G15" s="42">
+      <c r="G23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="H15" s="43">
-        <f>IF($C15=0,"",D15/$C15)</f>
-        <v/>
-      </c>
-      <c r="I15" s="43">
-        <f>IF($C15=0,"",E15/$C15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="43">
-        <f>IF($C15=0,"",F15/$C15)</f>
-        <v/>
-      </c>
-      <c r="K15" s="43">
-        <f>IF($C15=0,"",G15/$C15)</f>
-        <v/>
-      </c>
-      <c r="L15" s="42">
+      <c r="H23" s="43">
+        <f>IF($C23=0,"",D23/$C23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="43">
+        <f>IF($C23=0,"",E23/$C23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="43">
+        <f>IF($C23=0,"",F23/$C23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="43">
+        <f>IF($C23=0,"",G23/$C23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"สูง",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="M15" s="42">
+      <c r="M23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ปานกลาง",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="N15" s="42">
+      <c r="N23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ต่ำ",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="O15" s="42">
+      <c r="O23" s="42">
         <f>COUNTIFS('3_วิจัยและบริการวิชาการ'!$T$7:$T$91,"?*",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="P15" s="44">
+      <c r="P23" s="44">
         <f>SUMIFS('3_วิจัยและบริการวิชาการ'!$U$7:$U$91,'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="Q15" s="42">
+      <c r="Q23" s="42">
         <f>COUNTIF('3_วิจัยและบริการวิชาการ'!$W$7:$W$91,"✔ ครบ")</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="41" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
         <is>
           <t>งานบริการการศึกษาและพัฒนาคุณภาพนักศึกษา</t>
         </is>
       </c>
-      <c r="B16" s="42">
+      <c r="B24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$C$7:$C$91,"?*",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="C16" s="42">
+      <c r="C24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$C$7:$C$91,"?*",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"?*",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="D16" s="42">
+      <c r="D24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$P$7:$P$91,"คง D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="E16" s="42">
+      <c r="E24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ตัด D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="F16" s="42">
+      <c r="F24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="G16" s="42">
+      <c r="G24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="H16" s="43">
-        <f>IF($C16=0,"",D16/$C16)</f>
-        <v/>
-      </c>
-      <c r="I16" s="43">
-        <f>IF($C16=0,"",E16/$C16)</f>
-        <v/>
-      </c>
-      <c r="J16" s="43">
-        <f>IF($C16=0,"",F16/$C16)</f>
-        <v/>
-      </c>
-      <c r="K16" s="43">
-        <f>IF($C16=0,"",G16/$C16)</f>
-        <v/>
-      </c>
-      <c r="L16" s="42">
+      <c r="H24" s="43">
+        <f>IF($C24=0,"",D24/$C24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="43">
+        <f>IF($C24=0,"",E24/$C24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="43">
+        <f>IF($C24=0,"",F24/$C24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="43">
+        <f>IF($C24=0,"",G24/$C24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"สูง",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="M16" s="42">
+      <c r="M24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ปานกลาง",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="N16" s="42">
+      <c r="N24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ต่ำ",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="O16" s="42">
+      <c r="O24" s="42">
         <f>COUNTIFS('4_การศึกษาและนักศึกษา'!$T$7:$T$91,"?*",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="P16" s="44">
+      <c r="P24" s="44">
         <f>SUMIFS('4_การศึกษาและนักศึกษา'!$U$7:$U$91,'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="Q16" s="42">
+      <c r="Q24" s="42">
         <f>COUNTIF('4_การศึกษาและนักศึกษา'!$W$7:$W$91,"✔ ครบ")</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="45" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
         <is>
           <t>ทั้งคณะ</t>
         </is>
       </c>
-      <c r="B17" s="46">
-        <f>SUM(B13:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="46">
-        <f>SUM(C13:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="46">
-        <f>SUM(D13:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="46">
-        <f>SUM(E13:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="46">
-        <f>SUM(F13:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="46">
-        <f>SUM(G13:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="47">
-        <f>IF($C17=0,"",D17/$C17)</f>
-        <v/>
-      </c>
-      <c r="I17" s="47">
-        <f>IF($C17=0,"",E17/$C17)</f>
-        <v/>
-      </c>
-      <c r="J17" s="47">
-        <f>IF($C17=0,"",F17/$C17)</f>
-        <v/>
-      </c>
-      <c r="K17" s="47">
-        <f>IF($C17=0,"",G17/$C17)</f>
-        <v/>
-      </c>
-      <c r="L17" s="46">
-        <f>SUM(L13:L16)</f>
-        <v/>
-      </c>
-      <c r="M17" s="46">
-        <f>SUM(M13:M16)</f>
-        <v/>
-      </c>
-      <c r="N17" s="46">
-        <f>SUM(N13:N16)</f>
-        <v/>
-      </c>
-      <c r="O17" s="46">
-        <f>SUM(O13:O16)</f>
-        <v/>
-      </c>
-      <c r="P17" s="48">
-        <f>SUM(P13:P16)</f>
-        <v/>
-      </c>
-      <c r="Q17" s="46">
-        <f>SUM(Q13:Q16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="B25" s="46">
+        <f>SUM(B21:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="46">
+        <f>SUM(C21:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="46">
+        <f>SUM(D21:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="46">
+        <f>SUM(E21:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="46">
+        <f>SUM(F21:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="46">
+        <f>SUM(G21:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="47">
+        <f>IF($C25=0,"",D25/$C25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="47">
+        <f>IF($C25=0,"",E25/$C25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="47">
+        <f>IF($C25=0,"",F25/$C25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="47">
+        <f>IF($C25=0,"",G25/$C25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="46">
+        <f>SUM(L21:L24)</f>
+        <v/>
+      </c>
+      <c r="M25" s="46">
+        <f>SUM(M21:M24)</f>
+        <v/>
+      </c>
+      <c r="N25" s="46">
+        <f>SUM(N21:N24)</f>
+        <v/>
+      </c>
+      <c r="O25" s="46">
+        <f>SUM(O21:O24)</f>
+        <v/>
+      </c>
+      <c r="P25" s="48">
+        <f>SUM(P21:P24)</f>
+        <v/>
+      </c>
+      <c r="Q25" s="46">
+        <f>SUM(Q21:Q24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>ความเสี่ยง × ข้อเสนอ (ทั้งคณะ) — ใช้ดูว่าข้อเสนอสอดคล้องกับระดับความเสี่ยงหรือไม่</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>ระดับความเสี่ยง \ ข้อเสนอ</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>คง D2</t>
         </is>
       </c>
-      <c r="C20" s="16" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>ตัด D2</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>เปลี่ยนเป็น
 ผู้เชี่ยวชาญ</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>ขอหารือ
 เพิ่มเติม</t>
         </is>
       </c>
-      <c r="F20" s="16" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>รวม</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="41" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
         <is>
           <t>สูง</t>
         </is>
       </c>
-      <c r="B21" s="42">
+      <c r="B29" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"สูง",'1_บริหารทั่วไป'!$P$7:$P$91,"คง D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"สูง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"คง D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"สูง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"คง D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"สูง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"คง D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="C21" s="42">
+      <c r="C29" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"สูง",'1_บริหารทั่วไป'!$P$7:$P$91,"ตัด D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"สูง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ตัด D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"สูง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ตัด D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"สูง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ตัด D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="D21" s="42">
+      <c r="D29" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"สูง",'1_บริหารทั่วไป'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"สูง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"สูง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"สูง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="E21" s="42">
+      <c r="E29" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"สูง",'1_บริหารทั่วไป'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"สูง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"สูง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"สูง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="F21" s="49">
-        <f>SUM(B21:E21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="41" t="inlineStr">
+      <c r="F29" s="49">
+        <f>SUM(B29:E29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="41" t="inlineStr">
         <is>
           <t>ปานกลาง</t>
         </is>
       </c>
-      <c r="B22" s="42">
+      <c r="B30" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ปานกลาง",'1_บริหารทั่วไป'!$P$7:$P$91,"คง D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ปานกลาง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"คง D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ปานกลาง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"คง D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ปานกลาง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"คง D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="C22" s="42">
+      <c r="C30" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ปานกลาง",'1_บริหารทั่วไป'!$P$7:$P$91,"ตัด D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ปานกลาง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ตัด D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ปานกลาง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ตัด D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ปานกลาง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ตัด D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="D22" s="42">
+      <c r="D30" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ปานกลาง",'1_บริหารทั่วไป'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ปานกลาง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ปานกลาง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ปานกลาง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="E22" s="42">
+      <c r="E30" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ปานกลาง",'1_บริหารทั่วไป'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ปานกลาง",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ปานกลาง",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ปานกลาง",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="F22" s="49">
-        <f>SUM(B22:E22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="41" t="inlineStr">
+      <c r="F30" s="49">
+        <f>SUM(B30:E30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="41" t="inlineStr">
         <is>
           <t>ต่ำ</t>
         </is>
       </c>
-      <c r="B23" s="42">
+      <c r="B31" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ต่ำ",'1_บริหารทั่วไป'!$P$7:$P$91,"คง D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ต่ำ",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"คง D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ต่ำ",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"คง D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ต่ำ",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"คง D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="C23" s="42">
+      <c r="C31" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ต่ำ",'1_บริหารทั่วไป'!$P$7:$P$91,"ตัด D2",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ต่ำ",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ตัด D2",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ต่ำ",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ตัด D2",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ต่ำ",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ตัด D2",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="D23" s="42">
+      <c r="D31" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ต่ำ",'1_บริหารทั่วไป'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ต่ำ",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ต่ำ",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ต่ำ",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"เปลี่ยนเป็นหน่วยงานผู้เชี่ยวชาญ",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="E23" s="42">
+      <c r="E31" s="42">
         <f>COUNTIFS('1_บริหารทั่วไป'!$S$7:$S$91,"ต่ำ",'1_บริหารทั่วไป'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'1_บริหารทั่วไป'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('2_ยุทธศาสตร์และแผน'!$S$7:$S$91,"ต่ำ",'2_ยุทธศาสตร์และแผน'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'2_ยุทธศาสตร์และแผน'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('3_วิจัยและบริการวิชาการ'!$S$7:$S$91,"ต่ำ",'3_วิจัยและบริการวิชาการ'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'3_วิจัยและบริการวิชาการ'!$D$7:$D$91,"&lt;&gt;0")+COUNTIFS('4_การศึกษาและนักศึกษา'!$S$7:$S$91,"ต่ำ",'4_การศึกษาและนักศึกษา'!$P$7:$P$91,"ขอหารือเพิ่มเติม",'4_การศึกษาและนักศึกษา'!$D$7:$D$91,"&lt;&gt;0")</f>
         <v/>
       </c>
-      <c r="F23" s="49">
-        <f>SUM(B23:E23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="50" t="inlineStr">
+      <c r="F31" s="49">
+        <f>SUM(B31:E31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="50" t="inlineStr">
         <is>
           <t>ช่องสีส้ม = เสี่ยงสูงแต่เสนอตัด D2 | ช่องสีเหลือง = เสี่ยงต่ำแต่เสนอคง D2 (ควรทบทวนเป็นพิเศษ)</t>
         </is>
@@ -2593,28 +2666,28 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="A11:P11"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="J17:K17"/>
   </mergeCells>
-  <conditionalFormatting sqref="A21:A23">
+  <conditionalFormatting sqref="A29:A31">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"สูง"</formula>
     </cfRule>
@@ -2625,18 +2698,18 @@
       <formula>"ต่ำ"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
+  <conditionalFormatting sqref="C29">
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>C21&gt;0</formula>
+      <formula>C29&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23">
+  <conditionalFormatting sqref="B31">
     <cfRule type="expression" priority="5" dxfId="4">
-      <formula>B23&gt;0</formula>
+      <formula>B31&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=Settings!$K$5:$K$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>